<commit_message>
n8n board refresh 2026-10-30T17:41:38Z
</commit_message>
<xml_diff>
--- a/app/reports/BBT_research.xlsx
+++ b/app/reports/BBT_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-29 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-30 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>51.02</v>
+        <v>51.52</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>30.69</v>
+        <v>30.39</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.662</v>
+        <v>0.695</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04994999885559082</v>
+        <v>0.04933000087738037</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>83816093.32029977</v>
+        <v>83816084.76472524</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>30.69</v>
+        <v>30.39</v>
       </c>
     </row>
     <row r="38">
@@ -1520,14 +1520,14 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>2572315904</v>
+        <v>2547170816</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>9.65</v>
+        <v>9.56</v>
       </c>
       <c r="E5" s="32" t="n"/>
       <c r="F5" s="32" t="n">
-        <v>3.1</v>
+        <v>3.12</v>
       </c>
     </row>
     <row r="6">
@@ -1542,12 +1542,12 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>754310848</v>
+        <v>752114944</v>
       </c>
       <c r="D6" s="34" t="n"/>
       <c r="E6" s="34" t="n"/>
       <c r="F6" s="34" t="n">
-        <v>-2.02</v>
+        <v>-2.036</v>
       </c>
     </row>
     <row r="7">
@@ -1562,12 +1562,12 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>345162912</v>
+        <v>352478496</v>
       </c>
       <c r="D7" s="34" t="n"/>
       <c r="E7" s="34" t="n"/>
       <c r="F7" s="34" t="n">
-        <v>4.222</v>
+        <v>4.236</v>
       </c>
     </row>
     <row r="8">
@@ -1582,14 +1582,14 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>2238262784</v>
+        <v>2207675136</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>12.538076</v>
+        <v>12.366734</v>
       </c>
       <c r="E8" s="34" t="n"/>
       <c r="F8" s="34" t="n">
-        <v>3.295</v>
+        <v>3.297</v>
       </c>
     </row>
     <row r="9">
@@ -1604,16 +1604,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>754909440</v>
+        <v>771413504</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>23.750002</v>
+        <v>24.269232</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>7.047</v>
+        <v>7.196</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>1.977</v>
+        <v>2.019</v>
       </c>
     </row>
     <row r="10">
@@ -1628,16 +1628,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>11230622720</v>
+        <v>11087428608</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>24.954544</v>
+        <v>24.636364</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>20.859</v>
+        <v>20.978</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>1.918</v>
+        <v>1.929</v>
       </c>
     </row>
     <row r="11">
@@ -1652,16 +1652,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>1515592960</v>
+        <v>1489588224</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>21.686047</v>
+        <v>21.313953</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>9.58</v>
+        <v>9.537000000000001</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>4.281</v>
+        <v>4.262</v>
       </c>
     </row>
     <row r="12">
@@ -1676,16 +1676,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>2744261376</v>
+        <v>2600029696</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>26.13848</v>
+        <v>24.764706</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>17.951</v>
+        <v>17.717</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>6.522</v>
+        <v>6.437</v>
       </c>
     </row>
     <row r="13">
@@ -1700,14 +1700,14 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>1670411776</v>
+        <v>1678515840</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>18.83871</v>
+        <v>18.930107</v>
       </c>
       <c r="E13" s="34" t="n"/>
       <c r="F13" s="34" t="n">
-        <v>8.369999999999999</v>
+        <v>8.44</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-31T17:41:49Z
</commit_message>
<xml_diff>
--- a/app/reports/BBT_research.xlsx
+++ b/app/reports/BBT_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-30 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-31 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>51.52</v>
+        <v>51.56</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>30.39</v>
+        <v>30.62</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.695</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04933000087738037</v>
+        <v>0.04928999900817871</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>83816084.76472524</v>
+        <v>83816088.83082952</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>30.39</v>
+        <v>30.62</v>
       </c>
     </row>
     <row r="38">
@@ -1520,10 +1520,10 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>2547170816</v>
+        <v>2566448640</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>9.56</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="E5" s="32" t="n"/>
       <c r="F5" s="32" t="n">
@@ -1542,12 +1542,12 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>752114944</v>
+        <v>746625088</v>
       </c>
       <c r="D6" s="34" t="n"/>
       <c r="E6" s="34" t="n"/>
       <c r="F6" s="34" t="n">
-        <v>-2.036</v>
+        <v>-2.023</v>
       </c>
     </row>
     <row r="7">
@@ -1567,7 +1567,7 @@
       <c r="D7" s="34" t="n"/>
       <c r="E7" s="34" t="n"/>
       <c r="F7" s="34" t="n">
-        <v>4.236</v>
+        <v>4.244</v>
       </c>
     </row>
     <row r="8">
@@ -1582,14 +1582,14 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>2207675136</v>
+        <v>2211252736</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>12.366734</v>
+        <v>12.386774</v>
       </c>
       <c r="E8" s="34" t="n"/>
       <c r="F8" s="34" t="n">
-        <v>3.297</v>
+        <v>3.263</v>
       </c>
     </row>
     <row r="9">
@@ -1604,16 +1604,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>771413504</v>
+        <v>772636032</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>24.269232</v>
+        <v>24.307693</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>7.196</v>
+        <v>7.208</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>2.019</v>
+        <v>2.022</v>
       </c>
     </row>
     <row r="10">
@@ -1634,10 +1634,10 @@
         <v>24.636364</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>20.978</v>
+        <v>20.383</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>1.929</v>
+        <v>1.874</v>
       </c>
     </row>
     <row r="11">
@@ -1652,16 +1652,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>1489588224</v>
+        <v>1492026240</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>21.313953</v>
+        <v>21.348837</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>9.537000000000001</v>
+        <v>9.435</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>4.262</v>
+        <v>4.217</v>
       </c>
     </row>
     <row r="12">
@@ -1676,16 +1676,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>2600029696</v>
+        <v>2600801792</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>24.764706</v>
+        <v>24.772058</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>17.717</v>
+        <v>16.728</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>6.437</v>
+        <v>6.077</v>
       </c>
     </row>
     <row r="13">
@@ -1700,14 +1700,14 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>1678515840</v>
+        <v>1680899456</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>18.930107</v>
+        <v>18.956987</v>
       </c>
       <c r="E13" s="34" t="n"/>
       <c r="F13" s="34" t="n">
-        <v>8.44</v>
+        <v>8.442</v>
       </c>
     </row>
     <row r="15">

</xml_diff>